<commit_message>
botao de visualizar pins de bricks
</commit_message>
<xml_diff>
--- a/CP Mafra.xlsx
+++ b/CP Mafra.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\Apps\Classifica Pack\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\Apps\Classifica Pack DEV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41782D68-6268-4E0B-B936-5498E8D6AE59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A9BAB3F-B704-4643-AF12-C46EDB0BDECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="864" activeTab="8" xr2:uid="{99CD96B6-2742-484F-A436-0F4B0ADED557}"/>
   </bookViews>
@@ -1165,7 +1165,7 @@
         <v>97</v>
       </c>
       <c r="E1" t="str">
-        <f>B1 &amp; "-" &amp; TEXT(C1, "000")</f>
+        <f t="shared" ref="E1:E32" si="0">B1 &amp; "-" &amp; TEXT(C1, "000")</f>
         <v>2665-004</v>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
         <v>97</v>
       </c>
       <c r="E2" t="str">
-        <f>B2 &amp; "-" &amp; TEXT(C2, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-020</v>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
         <v>97</v>
       </c>
       <c r="E3" t="str">
-        <f>B3 &amp; "-" &amp; TEXT(C3, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-012</v>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
         <v>97</v>
       </c>
       <c r="E4" t="str">
-        <f>B4 &amp; "-" &amp; TEXT(C4, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-004</v>
       </c>
     </row>
@@ -1237,7 +1237,7 @@
         <v>97</v>
       </c>
       <c r="E5" t="str">
-        <f>B5 &amp; "-" &amp; TEXT(C5, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-022</v>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
         <v>97</v>
       </c>
       <c r="E6" t="str">
-        <f>B6 &amp; "-" &amp; TEXT(C6, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-012</v>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
         <v>97</v>
       </c>
       <c r="E7" t="str">
-        <f>B7 &amp; "-" &amp; TEXT(C7, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-017</v>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
         <v>97</v>
       </c>
       <c r="E8" t="str">
-        <f>B8 &amp; "-" &amp; TEXT(C8, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-017</v>
       </c>
     </row>
@@ -1309,7 +1309,7 @@
         <v>97</v>
       </c>
       <c r="E9" t="str">
-        <f>B9 &amp; "-" &amp; TEXT(C9, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-004</v>
       </c>
     </row>
@@ -1327,7 +1327,7 @@
         <v>97</v>
       </c>
       <c r="E10" t="str">
-        <f>B10 &amp; "-" &amp; TEXT(C10, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-022</v>
       </c>
     </row>
@@ -1345,7 +1345,7 @@
         <v>97</v>
       </c>
       <c r="E11" t="str">
-        <f>B11 &amp; "-" &amp; TEXT(C11, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-003</v>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
         <v>97</v>
       </c>
       <c r="E12" t="str">
-        <f>B12 &amp; "-" &amp; TEXT(C12, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-003</v>
       </c>
     </row>
@@ -1381,7 +1381,7 @@
         <v>97</v>
       </c>
       <c r="E13" t="str">
-        <f>B13 &amp; "-" &amp; TEXT(C13, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-004</v>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
         <v>97</v>
       </c>
       <c r="E14" t="str">
-        <f>B14 &amp; "-" &amp; TEXT(C14, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-003</v>
       </c>
     </row>
@@ -1417,7 +1417,7 @@
         <v>97</v>
       </c>
       <c r="E15" t="str">
-        <f>B15 &amp; "-" &amp; TEXT(C15, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-003</v>
       </c>
     </row>
@@ -1435,7 +1435,7 @@
         <v>97</v>
       </c>
       <c r="E16" t="str">
-        <f>B16 &amp; "-" &amp; TEXT(C16, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-017</v>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
         <v>97</v>
       </c>
       <c r="E17" t="str">
-        <f>B17 &amp; "-" &amp; TEXT(C17, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-017</v>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
         <v>97</v>
       </c>
       <c r="E18" t="str">
-        <f>B18 &amp; "-" &amp; TEXT(C18, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-004</v>
       </c>
     </row>
@@ -1489,7 +1489,7 @@
         <v>97</v>
       </c>
       <c r="E19" t="str">
-        <f>B19 &amp; "-" &amp; TEXT(C19, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-004</v>
       </c>
     </row>
@@ -1507,7 +1507,7 @@
         <v>97</v>
       </c>
       <c r="E20" t="str">
-        <f>B20 &amp; "-" &amp; TEXT(C20, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-004</v>
       </c>
     </row>
@@ -1525,7 +1525,7 @@
         <v>97</v>
       </c>
       <c r="E21" t="str">
-        <f>B21 &amp; "-" &amp; TEXT(C21, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-004</v>
       </c>
     </row>
@@ -1543,7 +1543,7 @@
         <v>97</v>
       </c>
       <c r="E22" t="str">
-        <f>B22 &amp; "-" &amp; TEXT(C22, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-004</v>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
         <v>97</v>
       </c>
       <c r="E23" t="str">
-        <f>B23 &amp; "-" &amp; TEXT(C23, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-004</v>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
         <v>97</v>
       </c>
       <c r="E24" t="str">
-        <f>B24 &amp; "-" &amp; TEXT(C24, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-022</v>
       </c>
     </row>
@@ -1597,7 +1597,7 @@
         <v>97</v>
       </c>
       <c r="E25" t="str">
-        <f>B25 &amp; "-" &amp; TEXT(C25, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-022</v>
       </c>
     </row>
@@ -1615,7 +1615,7 @@
         <v>97</v>
       </c>
       <c r="E26" t="str">
-        <f>B26 &amp; "-" &amp; TEXT(C26, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-011</v>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
         <v>97</v>
       </c>
       <c r="E27" t="str">
-        <f>B27 &amp; "-" &amp; TEXT(C27, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-017</v>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
         <v>97</v>
       </c>
       <c r="E28" t="str">
-        <f>B28 &amp; "-" &amp; TEXT(C28, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-004</v>
       </c>
     </row>
@@ -1669,7 +1669,7 @@
         <v>97</v>
       </c>
       <c r="E29" t="str">
-        <f>B29 &amp; "-" &amp; TEXT(C29, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-008</v>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
         <v>97</v>
       </c>
       <c r="E30" t="str">
-        <f>B30 &amp; "-" &amp; TEXT(C30, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-010</v>
       </c>
     </row>
@@ -1705,7 +1705,7 @@
         <v>97</v>
       </c>
       <c r="E31" t="str">
-        <f>B31 &amp; "-" &amp; TEXT(C31, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-011</v>
       </c>
     </row>
@@ -1723,7 +1723,7 @@
         <v>97</v>
       </c>
       <c r="E32" t="str">
-        <f>B32 &amp; "-" &amp; TEXT(C32, "000")</f>
+        <f t="shared" si="0"/>
         <v>2665-013</v>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
         <v>97</v>
       </c>
       <c r="E33" t="str">
-        <f>B33 &amp; "-" &amp; TEXT(C33, "000")</f>
+        <f t="shared" ref="E33:E64" si="1">B33 &amp; "-" &amp; TEXT(C33, "000")</f>
         <v>2665-018</v>
       </c>
     </row>
@@ -1759,7 +1759,7 @@
         <v>97</v>
       </c>
       <c r="E34" t="str">
-        <f>B34 &amp; "-" &amp; TEXT(C34, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-018</v>
       </c>
     </row>
@@ -1777,7 +1777,7 @@
         <v>97</v>
       </c>
       <c r="E35" t="str">
-        <f>B35 &amp; "-" &amp; TEXT(C35, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-018</v>
       </c>
     </row>
@@ -1795,7 +1795,7 @@
         <v>97</v>
       </c>
       <c r="E36" t="str">
-        <f>B36 &amp; "-" &amp; TEXT(C36, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-018</v>
       </c>
     </row>
@@ -1813,7 +1813,7 @@
         <v>97</v>
       </c>
       <c r="E37" t="str">
-        <f>B37 &amp; "-" &amp; TEXT(C37, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-018</v>
       </c>
     </row>
@@ -1831,7 +1831,7 @@
         <v>97</v>
       </c>
       <c r="E38" t="str">
-        <f>B38 &amp; "-" &amp; TEXT(C38, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-018</v>
       </c>
     </row>
@@ -1849,7 +1849,7 @@
         <v>97</v>
       </c>
       <c r="E39" t="str">
-        <f>B39 &amp; "-" &amp; TEXT(C39, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-018</v>
       </c>
     </row>
@@ -1867,7 +1867,7 @@
         <v>97</v>
       </c>
       <c r="E40" t="str">
-        <f>B40 &amp; "-" &amp; TEXT(C40, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-018</v>
       </c>
     </row>
@@ -1885,7 +1885,7 @@
         <v>97</v>
       </c>
       <c r="E41" t="str">
-        <f>B41 &amp; "-" &amp; TEXT(C41, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-018</v>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
         <v>97</v>
       </c>
       <c r="E42" t="str">
-        <f>B42 &amp; "-" &amp; TEXT(C42, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-002</v>
       </c>
     </row>
@@ -1921,7 +1921,7 @@
         <v>97</v>
       </c>
       <c r="E43" t="str">
-        <f>B43 &amp; "-" &amp; TEXT(C43, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-002</v>
       </c>
     </row>
@@ -1939,7 +1939,7 @@
         <v>97</v>
       </c>
       <c r="E44" t="str">
-        <f>B44 &amp; "-" &amp; TEXT(C44, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-002</v>
       </c>
     </row>
@@ -1957,7 +1957,7 @@
         <v>97</v>
       </c>
       <c r="E45" t="str">
-        <f>B45 &amp; "-" &amp; TEXT(C45, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-002</v>
       </c>
     </row>
@@ -1975,7 +1975,7 @@
         <v>97</v>
       </c>
       <c r="E46" t="str">
-        <f>B46 &amp; "-" &amp; TEXT(C46, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-997</v>
       </c>
     </row>
@@ -1993,7 +1993,7 @@
         <v>97</v>
       </c>
       <c r="E47" t="str">
-        <f>B47 &amp; "-" &amp; TEXT(C47, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-015</v>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
         <v>97</v>
       </c>
       <c r="E48" t="str">
-        <f>B48 &amp; "-" &amp; TEXT(C48, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-009</v>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
         <v>97</v>
       </c>
       <c r="E49" t="str">
-        <f>B49 &amp; "-" &amp; TEXT(C49, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2047,7 +2047,7 @@
         <v>97</v>
       </c>
       <c r="E50" t="str">
-        <f>B50 &amp; "-" &amp; TEXT(C50, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2065,7 +2065,7 @@
         <v>97</v>
       </c>
       <c r="E51" t="str">
-        <f>B51 &amp; "-" &amp; TEXT(C51, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2083,7 +2083,7 @@
         <v>97</v>
       </c>
       <c r="E52" t="str">
-        <f>B52 &amp; "-" &amp; TEXT(C52, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
         <v>97</v>
       </c>
       <c r="E53" t="str">
-        <f>B53 &amp; "-" &amp; TEXT(C53, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
         <v>97</v>
       </c>
       <c r="E54" t="str">
-        <f>B54 &amp; "-" &amp; TEXT(C54, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2137,7 +2137,7 @@
         <v>97</v>
       </c>
       <c r="E55" t="str">
-        <f>B55 &amp; "-" &amp; TEXT(C55, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2155,7 +2155,7 @@
         <v>97</v>
       </c>
       <c r="E56" t="str">
-        <f>B56 &amp; "-" &amp; TEXT(C56, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2173,7 +2173,7 @@
         <v>97</v>
       </c>
       <c r="E57" t="str">
-        <f>B57 &amp; "-" &amp; TEXT(C57, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2191,7 +2191,7 @@
         <v>97</v>
       </c>
       <c r="E58" t="str">
-        <f>B58 &amp; "-" &amp; TEXT(C58, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2209,7 +2209,7 @@
         <v>97</v>
       </c>
       <c r="E59" t="str">
-        <f>B59 &amp; "-" &amp; TEXT(C59, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2227,7 +2227,7 @@
         <v>97</v>
       </c>
       <c r="E60" t="str">
-        <f>B60 &amp; "-" &amp; TEXT(C60, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2245,7 +2245,7 @@
         <v>97</v>
       </c>
       <c r="E61" t="str">
-        <f>B61 &amp; "-" &amp; TEXT(C61, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
         <v>97</v>
       </c>
       <c r="E62" t="str">
-        <f>B62 &amp; "-" &amp; TEXT(C62, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2281,7 +2281,7 @@
         <v>97</v>
       </c>
       <c r="E63" t="str">
-        <f>B63 &amp; "-" &amp; TEXT(C63, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2299,7 +2299,7 @@
         <v>97</v>
       </c>
       <c r="E64" t="str">
-        <f>B64 &amp; "-" &amp; TEXT(C64, "000")</f>
+        <f t="shared" si="1"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2317,7 +2317,7 @@
         <v>97</v>
       </c>
       <c r="E65" t="str">
-        <f>B65 &amp; "-" &amp; TEXT(C65, "000")</f>
+        <f t="shared" ref="E65:E94" si="2">B65 &amp; "-" &amp; TEXT(C65, "000")</f>
         <v>2665-006</v>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
         <v>97</v>
       </c>
       <c r="E66" t="str">
-        <f>B66 &amp; "-" &amp; TEXT(C66, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2353,7 +2353,7 @@
         <v>97</v>
       </c>
       <c r="E67" t="str">
-        <f>B67 &amp; "-" &amp; TEXT(C67, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2371,7 +2371,7 @@
         <v>97</v>
       </c>
       <c r="E68" t="str">
-        <f>B68 &amp; "-" &amp; TEXT(C68, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-006</v>
       </c>
     </row>
@@ -2389,7 +2389,7 @@
         <v>97</v>
       </c>
       <c r="E69" t="str">
-        <f>B69 &amp; "-" &amp; TEXT(C69, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-020</v>
       </c>
     </row>
@@ -2407,7 +2407,7 @@
         <v>97</v>
       </c>
       <c r="E70" t="str">
-        <f>B70 &amp; "-" &amp; TEXT(C70, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2425,7 +2425,7 @@
         <v>97</v>
       </c>
       <c r="E71" t="str">
-        <f>B71 &amp; "-" &amp; TEXT(C71, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-022</v>
       </c>
     </row>
@@ -2443,7 +2443,7 @@
         <v>97</v>
       </c>
       <c r="E72" t="str">
-        <f>B72 &amp; "-" &amp; TEXT(C72, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-022</v>
       </c>
     </row>
@@ -2461,7 +2461,7 @@
         <v>97</v>
       </c>
       <c r="E73" t="str">
-        <f>B73 &amp; "-" &amp; TEXT(C73, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-022</v>
       </c>
     </row>
@@ -2479,7 +2479,7 @@
         <v>97</v>
       </c>
       <c r="E74" t="str">
-        <f>B74 &amp; "-" &amp; TEXT(C74, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2497,7 +2497,7 @@
         <v>97</v>
       </c>
       <c r="E75" t="str">
-        <f>B75 &amp; "-" &amp; TEXT(C75, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2515,7 +2515,7 @@
         <v>97</v>
       </c>
       <c r="E76" t="str">
-        <f>B76 &amp; "-" &amp; TEXT(C76, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2533,7 +2533,7 @@
         <v>97</v>
       </c>
       <c r="E77" t="str">
-        <f>B77 &amp; "-" &amp; TEXT(C77, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
         <v>97</v>
       </c>
       <c r="E78" t="str">
-        <f>B78 &amp; "-" &amp; TEXT(C78, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2569,7 +2569,7 @@
         <v>97</v>
       </c>
       <c r="E79" t="str">
-        <f>B79 &amp; "-" &amp; TEXT(C79, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2587,7 +2587,7 @@
         <v>97</v>
       </c>
       <c r="E80" t="str">
-        <f>B80 &amp; "-" &amp; TEXT(C80, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2605,7 +2605,7 @@
         <v>97</v>
       </c>
       <c r="E81" t="str">
-        <f>B81 &amp; "-" &amp; TEXT(C81, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2623,7 +2623,7 @@
         <v>97</v>
       </c>
       <c r="E82" t="str">
-        <f>B82 &amp; "-" &amp; TEXT(C82, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2641,7 +2641,7 @@
         <v>97</v>
       </c>
       <c r="E83" t="str">
-        <f>B83 &amp; "-" &amp; TEXT(C83, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2659,7 +2659,7 @@
         <v>97</v>
       </c>
       <c r="E84" t="str">
-        <f>B84 &amp; "-" &amp; TEXT(C84, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2677,7 +2677,7 @@
         <v>97</v>
       </c>
       <c r="E85" t="str">
-        <f>B85 &amp; "-" &amp; TEXT(C85, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2695,7 +2695,7 @@
         <v>97</v>
       </c>
       <c r="E86" t="str">
-        <f>B86 &amp; "-" &amp; TEXT(C86, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2713,7 +2713,7 @@
         <v>97</v>
       </c>
       <c r="E87" t="str">
-        <f>B87 &amp; "-" &amp; TEXT(C87, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2731,7 +2731,7 @@
         <v>97</v>
       </c>
       <c r="E88" t="str">
-        <f>B88 &amp; "-" &amp; TEXT(C88, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2749,7 +2749,7 @@
         <v>97</v>
       </c>
       <c r="E89" t="str">
-        <f>B89 &amp; "-" &amp; TEXT(C89, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2767,7 +2767,7 @@
         <v>97</v>
       </c>
       <c r="E90" t="str">
-        <f>B90 &amp; "-" &amp; TEXT(C90, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-007</v>
       </c>
     </row>
@@ -2785,7 +2785,7 @@
         <v>97</v>
       </c>
       <c r="E91" t="str">
-        <f>B91 &amp; "-" &amp; TEXT(C91, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-001</v>
       </c>
     </row>
@@ -2803,7 +2803,7 @@
         <v>97</v>
       </c>
       <c r="E92" t="str">
-        <f>B92 &amp; "-" &amp; TEXT(C92, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-003</v>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
         <v>97</v>
       </c>
       <c r="E93" t="str">
-        <f>B93 &amp; "-" &amp; TEXT(C93, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-005</v>
       </c>
     </row>
@@ -2839,7 +2839,7 @@
         <v>97</v>
       </c>
       <c r="E94" t="str">
-        <f>B94 &amp; "-" &amp; TEXT(C94, "000")</f>
+        <f t="shared" si="2"/>
         <v>2665-014</v>
       </c>
     </row>

</xml_diff>